<commit_message>
Refresh repository with full operational risk workflow
</commit_message>
<xml_diff>
--- a/data/processed/jfk_airline_delay_core_cleaned.xlsx
+++ b/data/processed/jfk_airline_delay_core_cleaned.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,67 +429,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>airline_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>total_arrival_flights</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>cancelled_arrivals</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>diverted_arrivals</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>delayed_arrivals_15_plus</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>total_arrival_delay_minutes</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>airline_delay_minutes</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>weather_delay_minutes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>nas_delay_minutes</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>security_delay_minutes</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>late_aircraft_delay_minutes</t>
         </is>
@@ -4835,7 +4847,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5179,7 +5191,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -5566,7 +5578,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -5910,7 +5922,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6254,7 +6266,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -6598,7 +6610,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -6942,7 +6954,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -7286,7 +7298,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -7630,7 +7642,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -7974,7 +7986,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -8318,7 +8330,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -8662,7 +8674,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -9006,7 +9018,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -9350,7 +9362,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D208" t="n">
@@ -9694,7 +9706,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -10038,7 +10050,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -10382,7 +10394,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D232" t="n">
@@ -10726,7 +10738,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -11070,7 +11082,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -11414,7 +11426,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>United Airlines</t>
+          <t>United Air Lines Network</t>
         </is>
       </c>
       <c r="D256" t="n">

</xml_diff>